<commit_message>
Update negative price analysis 2026-03
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Audit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update pipeline outputs Apr 2026
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3304,6 +3304,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3315,7 +3349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6170,8 +6204,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B83">
+  <conditionalFormatting sqref="B2:B84">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6183,7 +6251,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C83">
+  <conditionalFormatting sqref="C2:C84">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6195,7 +6263,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D83">
+  <conditionalFormatting sqref="D2:D84">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6207,7 +6275,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E83">
+  <conditionalFormatting sqref="E2:E84">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6219,7 +6287,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F83">
+  <conditionalFormatting sqref="F2:F84">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6231,7 +6299,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G83">
+  <conditionalFormatting sqref="G2:G84">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6243,7 +6311,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H83">
+  <conditionalFormatting sqref="H2:H84">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6255,7 +6323,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I83">
+  <conditionalFormatting sqref="I2:I84">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6267,7 +6335,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J83">
+  <conditionalFormatting sqref="J2:J84">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6289,7 +6357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9396,6 +9464,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>402</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update negative price analysis 2026-08 (logic-pass rewrite)
Full refresh, 2019-05..2026-08, run with --allow-history-rewrite "logic pass 2026-10: H1
interval-start daylight window, M1 cent-rounded thresholds".
- H1: daylight is now intervals STARTING 08:00-15:55 (it was intervals ending 08:00-15:55, i.e.
  07:55-15:55): QLD1 2023-10 81.45% → 80.65%
- M1: prices compared at whole cents, so solver noise like −$0.00002 no longer counts as below $0:
  QLD1 2026-01 25.30% → 21.37% (both fixes), VIC1 2020-03 2.35% → 0.67%
1,514 of 3,960 count cells and 363 of 440 rows change; totals unchanged. summary.csv is
byte-identical to an independent recompute from the raw DISPATCHPRICE archives. The exact
validator passes; page gates 36/0 and 45/0 on this data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0</v>
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0</v>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0.1</v>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.52</v>
+        <v>0.31</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>0.17</v>
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>0.1</v>
@@ -795,10 +795,10 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.1</v>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>0</v>
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>0</v>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2.47</v>
+        <v>1.6</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>1.25</v>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.34</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0.13</v>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.52</v>
+        <v>0.03</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0.03</v>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>0.13</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C24" s="3" t="n">
         <v>0</v>
@@ -1305,7 +1305,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>4.72</v>
+        <v>4.13</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>2.6</v>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.44</v>
+        <v>0.24</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>0.17</v>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>0.03</v>
@@ -1407,31 +1407,31 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2.92</v>
+        <v>2.65</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1.48</v>
+        <v>1.44</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29">
@@ -1441,19 +1441,19 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>13.61</v>
+        <v>13.58</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>8.77</v>
+        <v>8.74</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>6.38</v>
+        <v>6.35</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>4.2</v>
+        <v>4.17</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>1.71</v>
+        <v>1.68</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>1.21</v>
@@ -1475,16 +1475,16 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>27.12</v>
+        <v>26.6</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>18.75</v>
+        <v>18.68</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>14.27</v>
+        <v>14.2</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>10.56</v>
+        <v>10.52</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>2.57</v>
@@ -1509,10 +1509,10 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>24.26</v>
+        <v>24.06</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>19.89</v>
+        <v>19.86</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>18.08</v>
@@ -1543,16 +1543,16 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>8.19</v>
+        <v>7.85</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>6.91</v>
+        <v>6.88</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>5.73</v>
+        <v>5.69</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>5.14</v>
+        <v>5.1</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.97</v>
@@ -1577,13 +1577,13 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>4.47</v>
+        <v>4.37</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>3.02</v>
+        <v>2.92</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>2.52</v>
+        <v>2.49</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>2.45</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>0.24</v>
@@ -1645,10 +1645,10 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>3.42</v>
+        <v>3.27</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>2.27</v>
+        <v>2.23</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>1.97</v>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="C36" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>0.14</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="C39" s="3" t="n">
         <v>0.59</v>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>1.68</v>
+        <v>1.38</v>
       </c>
       <c r="C40" s="3" t="n">
         <v>0.9399999999999999</v>
@@ -1849,13 +1849,13 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>7.29</v>
+        <v>7.12</v>
       </c>
       <c r="C41" s="3" t="n">
         <v>5.71</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>5.28</v>
+        <v>5.24</v>
       </c>
       <c r="E41" s="3" t="n">
         <v>4.7</v>
@@ -1883,10 +1883,10 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>18.78</v>
+        <v>18.61</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>16.18</v>
+        <v>16.11</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>14.83</v>
@@ -1901,10 +1901,10 @@
         <v>5.8</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>2.29</v>
+        <v>2.26</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="J42" s="3" t="n">
         <v>0</v>
@@ -1917,25 +1917,25 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>11.83</v>
+        <v>11.73</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>10.32</v>
+        <v>10.25</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>9.109999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>8.4</v>
+        <v>8.33</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>6.79</v>
+        <v>6.72</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>5.14</v>
+        <v>5.07</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>4.03</v>
+        <v>3.97</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>1.01</v>
@@ -1951,25 +1951,25 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>20.59</v>
+        <v>20.38</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>15.07</v>
+        <v>14.93</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>13.51</v>
+        <v>13.4</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>11.63</v>
+        <v>11.56</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>9.17</v>
+        <v>9.1</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>6.25</v>
+        <v>6.22</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>3.16</v>
+        <v>3.09</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.38</v>
@@ -1985,22 +1985,22 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>32.83</v>
+        <v>32.49</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>22.11</v>
+        <v>21.81</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>19.46</v>
+        <v>19.15</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>16.53</v>
+        <v>16.33</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>12.63</v>
+        <v>12.47</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>8.43</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>1.88</v>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>7.83</v>
+        <v>7.69</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>6.08</v>
+        <v>5.95</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>5.65</v>
+        <v>5.51</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>5.11</v>
+        <v>5.04</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>3.8</v>
+        <v>3.73</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>2.15</v>
+        <v>2.08</v>
       </c>
       <c r="H46" s="3" t="n">
         <v>0.17</v>
@@ -2056,19 +2056,19 @@
         <v>10.68</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>7.51</v>
+        <v>7.59</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>7.22</v>
+        <v>7.29</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>6.96</v>
+        <v>7.03</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>6.32</v>
+        <v>6.36</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>3.83</v>
+        <v>3.87</v>
       </c>
       <c r="H47" s="3" t="n">
         <v>0.67</v>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>6.22</v>
+        <v>5.95</v>
       </c>
       <c r="C48" s="3" t="n">
         <v>4.47</v>
@@ -2099,7 +2099,7 @@
         <v>3.09</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>0</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>13.58</v>
+        <v>13.51</v>
       </c>
       <c r="C49" s="3" t="n">
         <v>11.74</v>
@@ -2133,10 +2133,10 @@
         <v>9.859999999999999</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>7.36</v>
+        <v>7.29</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>4.03</v>
+        <v>3.99</v>
       </c>
       <c r="H49" s="3" t="n">
         <v>2.19</v>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>2.05</v>
+        <v>1.85</v>
       </c>
       <c r="C50" s="3" t="n">
         <v>1.34</v>
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>4.72</v>
+        <v>4.44</v>
       </c>
       <c r="C51" s="3" t="n">
         <v>3.58</v>
@@ -2201,7 +2201,7 @@
         <v>2.71</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>2.15</v>
+        <v>1.84</v>
       </c>
       <c r="G51" s="3" t="n">
         <v>0.03</v>
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>15.99</v>
+        <v>15.09</v>
       </c>
       <c r="C52" s="3" t="n">
         <v>12.6</v>
@@ -2235,7 +2235,7 @@
         <v>9.85</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="G52" s="3" t="n">
         <v>2.65</v>
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>17.61</v>
+        <v>17.41</v>
       </c>
       <c r="C53" s="3" t="n">
         <v>14.01</v>
@@ -2269,7 +2269,7 @@
         <v>8.9</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>6.42</v>
+        <v>6.18</v>
       </c>
       <c r="G53" s="3" t="n">
         <v>1.85</v>
@@ -2291,22 +2291,22 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>39.27</v>
+        <v>39.03</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>35.62</v>
+        <v>35.42</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>32.81</v>
+        <v>32.64</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>25.62</v>
+        <v>25.52</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>24.24</v>
+        <v>24.13</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>16.88</v>
+        <v>16.84</v>
       </c>
       <c r="H54" s="3" t="n">
         <v>3.3</v>
@@ -2325,22 +2325,22 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>49.13</v>
+        <v>48.76</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>45.83</v>
+        <v>45.6</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>42.81</v>
+        <v>42.54</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>34.71</v>
+        <v>34.48</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>31.59</v>
+        <v>31.38</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>15.93</v>
+        <v>15.66</v>
       </c>
       <c r="H55" s="3" t="n">
         <v>1.61</v>
@@ -2359,19 +2359,19 @@
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>17.4</v>
+        <v>17.26</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>14.65</v>
+        <v>14.51</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>12.99</v>
+        <v>12.88</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>8.4</v>
+        <v>8.33</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>4.31</v>
+        <v>4.27</v>
       </c>
       <c r="G56" s="3" t="n">
         <v>1.35</v>
@@ -2393,19 +2393,19 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>21.24</v>
+        <v>21.2</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>19.76</v>
+        <v>19.72</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>15.83</v>
+        <v>15.76</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>12.16</v>
+        <v>12.1</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>6.82</v>
+        <v>6.85</v>
       </c>
       <c r="G57" s="3" t="n">
         <v>0.47</v>
@@ -2427,10 +2427,10 @@
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>4.64</v>
+        <v>4.6</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>3.83</v>
+        <v>3.8</v>
       </c>
       <c r="D58" s="3" t="n">
         <v>2.89</v>
@@ -2442,16 +2442,16 @@
         <v>1.04</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="H58" s="3" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="I58" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="I58" s="3" t="n">
+      <c r="J58" s="3" t="n">
         <v>0.37</v>
-      </c>
-      <c r="J58" s="3" t="n">
-        <v>0.34</v>
       </c>
     </row>
     <row r="59">
@@ -2461,16 +2461,16 @@
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>6.97</v>
+        <v>6.9</v>
       </c>
       <c r="C59" s="3" t="n">
-        <v>5.46</v>
+        <v>5.42</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>3.2</v>
+        <v>3.16</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1.83</v>
+        <v>1.8</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0.72</v>
@@ -2495,13 +2495,13 @@
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>13.78</v>
+        <v>13.61</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>11.29</v>
+        <v>11.16</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>8.199999999999999</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>4.23</v>
@@ -2529,19 +2529,19 @@
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>16.98</v>
+        <v>16.81</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>13.09</v>
+        <v>12.92</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>8.02</v>
+        <v>7.99</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>4.41</v>
+        <v>4.38</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>3.37</v>
+        <v>3.33</v>
       </c>
       <c r="G61" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>5.42</v>
+        <v>5.35</v>
       </c>
       <c r="C63" s="3" t="n">
         <v>3.99</v>
@@ -2634,7 +2634,7 @@
         <v>9.74</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>8.33</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>5.58</v>
@@ -2665,19 +2665,19 @@
         </is>
       </c>
       <c r="B65" s="3" t="n">
-        <v>30.71</v>
+        <v>30.54</v>
       </c>
       <c r="C65" s="3" t="n">
-        <v>27.45</v>
+        <v>27.28</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>24.9</v>
+        <v>24.76</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>22.01</v>
+        <v>21.98</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>18.58</v>
+        <v>18.55</v>
       </c>
       <c r="G65" s="3" t="n">
         <v>6.42</v>
@@ -2699,16 +2699,16 @@
         </is>
       </c>
       <c r="B66" s="3" t="n">
-        <v>56.7</v>
+        <v>56.67</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>50.97</v>
+        <v>50.94</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>48.54</v>
+        <v>48.51</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>44.06</v>
+        <v>44.03</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>36.6</v>
@@ -2733,19 +2733,19 @@
         </is>
       </c>
       <c r="B67" s="3" t="n">
-        <v>36.86</v>
+        <v>36.83</v>
       </c>
       <c r="C67" s="3" t="n">
-        <v>35.79</v>
+        <v>35.72</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>34.71</v>
+        <v>34.64</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>30.78</v>
+        <v>30.68</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>21.98</v>
+        <v>21.91</v>
       </c>
       <c r="G67" s="3" t="n">
         <v>4.77</v>
@@ -2767,16 +2767,16 @@
         </is>
       </c>
       <c r="B68" s="3" t="n">
-        <v>20.49</v>
+        <v>20.38</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>19.06</v>
+        <v>19.03</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>16.94</v>
+        <v>16.91</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>13.09</v>
+        <v>13.06</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>2.19</v>
@@ -2801,19 +2801,19 @@
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>36.29</v>
+        <v>36.12</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>34.44</v>
+        <v>34.27</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>31.18</v>
+        <v>31.01</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>23.66</v>
+        <v>23.49</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>3.49</v>
+        <v>3.46</v>
       </c>
       <c r="G69" s="3" t="n">
         <v>0.1</v>
@@ -2835,16 +2835,16 @@
         </is>
       </c>
       <c r="B70" s="3" t="n">
-        <v>35.32</v>
+        <v>35.22</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>34.17</v>
+        <v>34.11</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>29.87</v>
+        <v>29.84</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>19.42</v>
+        <v>19.35</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>1.34</v>
@@ -2869,16 +2869,16 @@
         </is>
       </c>
       <c r="B71" s="3" t="n">
-        <v>33.56</v>
+        <v>33.15</v>
       </c>
       <c r="C71" s="3" t="n">
-        <v>32.07</v>
+        <v>31.85</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>29.72</v>
+        <v>29.58</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>17.97</v>
+        <v>17.82</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>2.38</v>
@@ -2903,16 +2903,16 @@
         </is>
       </c>
       <c r="B72" s="3" t="n">
-        <v>23.66</v>
+        <v>23.15</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>19.79</v>
+        <v>19.56</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>15.93</v>
+        <v>15.73</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.54</v>
+        <v>0.5</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0.1</v>
@@ -2937,16 +2937,16 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>30.52</v>
+        <v>30.03</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>26.6</v>
+        <v>26.39</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>21.84</v>
+        <v>21.7</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>4.65</v>
+        <v>4.55</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0</v>
@@ -2971,13 +2971,13 @@
         </is>
       </c>
       <c r="B74" s="3" t="n">
-        <v>19.96</v>
+        <v>19.56</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>17.91</v>
+        <v>17.84</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>11.66</v>
+        <v>11.63</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>0.03</v>
@@ -3005,10 +3005,10 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>7.99</v>
+        <v>7.85</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>6.46</v>
+        <v>6.42</v>
       </c>
       <c r="D75" s="3" t="n">
         <v>2.33</v>
@@ -3039,13 +3039,13 @@
         </is>
       </c>
       <c r="B76" s="3" t="n">
-        <v>15.66</v>
+        <v>15.52</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>11.76</v>
+        <v>11.69</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>1.75</v>
+        <v>1.71</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>0</v>
@@ -3073,10 +3073,10 @@
         </is>
       </c>
       <c r="B77" s="3" t="n">
-        <v>26.88</v>
+        <v>26.75</v>
       </c>
       <c r="C77" s="3" t="n">
-        <v>19.29</v>
+        <v>19.32</v>
       </c>
       <c r="D77" s="3" t="n">
         <v>1.58</v>
@@ -3107,10 +3107,10 @@
         </is>
       </c>
       <c r="B78" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>70.62</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>60.73</v>
+        <v>60.56</v>
       </c>
       <c r="D78" s="3" t="n">
         <v>15.49</v>
@@ -3141,10 +3141,10 @@
         </is>
       </c>
       <c r="B79" s="3" t="n">
-        <v>59.85</v>
+        <v>59.48</v>
       </c>
       <c r="C79" s="3" t="n">
-        <v>48.62</v>
+        <v>48.45</v>
       </c>
       <c r="D79" s="3" t="n">
         <v>17.27</v>
@@ -3175,31 +3175,31 @@
         </is>
       </c>
       <c r="B80" s="3" t="n">
-        <v>74.72</v>
+        <v>74.41</v>
       </c>
       <c r="C80" s="3" t="n">
-        <v>53.85</v>
+        <v>53.33</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>15.97</v>
+        <v>16.04</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>3.99</v>
+        <v>4.03</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>1.39</v>
+        <v>1.42</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="81">
@@ -3209,13 +3209,13 @@
         </is>
       </c>
       <c r="B81" s="3" t="n">
-        <v>49.97</v>
+        <v>48.89</v>
       </c>
       <c r="C81" s="3" t="n">
-        <v>23.12</v>
+        <v>22.88</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>7.02</v>
+        <v>6.99</v>
       </c>
       <c r="E81" s="3" t="n">
         <v>4.33</v>
@@ -3243,16 +3243,16 @@
         </is>
       </c>
       <c r="B82" s="3" t="n">
-        <v>18.04</v>
+        <v>16.3</v>
       </c>
       <c r="C82" s="3" t="n">
-        <v>2.65</v>
+        <v>2.69</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F82" s="3" t="n">
         <v>0.1</v>
@@ -3277,16 +3277,16 @@
         </is>
       </c>
       <c r="B83" s="3" t="n">
-        <v>10.04</v>
+        <v>10.12</v>
       </c>
       <c r="C83" s="3" t="n">
-        <v>1.6</v>
+        <v>1.64</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>0.04</v>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="B84" s="3" t="n">
-        <v>13.51</v>
+        <v>13.27</v>
       </c>
       <c r="C84" s="3" t="n">
         <v>0.27</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="B85" s="3" t="n">
-        <v>19.2</v>
+        <v>18.78</v>
       </c>
       <c r="C85" s="3" t="n">
         <v>2.15</v>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="B86" s="3" t="n">
-        <v>4.3</v>
+        <v>4.03</v>
       </c>
       <c r="C86" s="3" t="n">
         <v>0</v>
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="B87" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="C87" s="3" t="n">
         <v>0</v>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="B88" s="3" t="n">
-        <v>4.37</v>
+        <v>4.33</v>
       </c>
       <c r="C88" s="3" t="n">
         <v>0</v>
@@ -3481,7 +3481,7 @@
         </is>
       </c>
       <c r="B89" s="3" t="n">
-        <v>6.92</v>
+        <v>6.82</v>
       </c>
       <c r="C89" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0</v>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0</v>
@@ -3695,7 +3695,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0.1</v>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.52</v>
+        <v>0.31</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>0.17</v>
@@ -3763,7 +3763,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>0.1</v>
@@ -3865,10 +3865,10 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.1</v>
@@ -3899,7 +3899,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>0</v>
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>0</v>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2.47</v>
+        <v>1.6</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>1.25</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.34</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0.13</v>
@@ -4103,7 +4103,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.52</v>
+        <v>0.03</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0.03</v>
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>0.13</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C24" s="3" t="n">
         <v>0</v>
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>4.72</v>
+        <v>4.13</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>2.6</v>
@@ -4409,7 +4409,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.44</v>
+        <v>0.24</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>0.17</v>
@@ -4443,7 +4443,7 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>0.03</v>
@@ -4477,31 +4477,31 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2.92</v>
+        <v>2.65</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1.48</v>
+        <v>1.44</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29">
@@ -4511,19 +4511,19 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>13.61</v>
+        <v>13.58</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>8.77</v>
+        <v>8.74</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>6.38</v>
+        <v>6.35</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>4.2</v>
+        <v>4.17</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>1.71</v>
+        <v>1.68</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>1.21</v>
@@ -4545,16 +4545,16 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>27.12</v>
+        <v>26.6</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>18.75</v>
+        <v>18.68</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>14.27</v>
+        <v>14.2</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>10.56</v>
+        <v>10.52</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>2.57</v>
@@ -4579,10 +4579,10 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>24.26</v>
+        <v>24.06</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>19.89</v>
+        <v>19.86</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>18.08</v>
@@ -4613,16 +4613,16 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>8.19</v>
+        <v>7.85</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>6.91</v>
+        <v>6.88</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>5.73</v>
+        <v>5.69</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>5.14</v>
+        <v>5.1</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.97</v>
@@ -4647,13 +4647,13 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>4.47</v>
+        <v>4.37</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>3.02</v>
+        <v>2.92</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>2.52</v>
+        <v>2.49</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>2.45</v>
@@ -4681,7 +4681,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>0.24</v>
@@ -4715,10 +4715,10 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>3.42</v>
+        <v>3.27</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>2.27</v>
+        <v>2.23</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>1.97</v>
@@ -4749,7 +4749,7 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="C36" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -4783,7 +4783,7 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>0.14</v>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="C39" s="3" t="n">
         <v>0.59</v>
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>1.68</v>
+        <v>1.38</v>
       </c>
       <c r="C40" s="3" t="n">
         <v>0.9399999999999999</v>
@@ -4919,13 +4919,13 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>7.29</v>
+        <v>7.12</v>
       </c>
       <c r="C41" s="3" t="n">
         <v>5.71</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>5.28</v>
+        <v>5.24</v>
       </c>
       <c r="E41" s="3" t="n">
         <v>4.7</v>
@@ -4953,10 +4953,10 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>18.78</v>
+        <v>18.61</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>16.18</v>
+        <v>16.11</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>14.83</v>
@@ -4971,10 +4971,10 @@
         <v>5.8</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>2.29</v>
+        <v>2.26</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="J42" s="3" t="n">
         <v>0</v>
@@ -4987,25 +4987,25 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>11.83</v>
+        <v>11.73</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>10.32</v>
+        <v>10.25</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>9.109999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>8.4</v>
+        <v>8.33</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>6.79</v>
+        <v>6.72</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>5.14</v>
+        <v>5.07</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>4.03</v>
+        <v>3.97</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>1.01</v>
@@ -5021,25 +5021,25 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>20.59</v>
+        <v>20.38</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>15.07</v>
+        <v>14.93</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>13.51</v>
+        <v>13.4</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>11.63</v>
+        <v>11.56</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>9.17</v>
+        <v>9.1</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>6.25</v>
+        <v>6.22</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>3.16</v>
+        <v>3.09</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.38</v>
@@ -5055,22 +5055,22 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>32.83</v>
+        <v>32.49</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>22.11</v>
+        <v>21.81</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>19.46</v>
+        <v>19.15</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>16.53</v>
+        <v>16.33</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>12.63</v>
+        <v>12.47</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>8.43</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>1.88</v>
@@ -5089,22 +5089,22 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>7.83</v>
+        <v>7.69</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>6.08</v>
+        <v>5.95</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>5.65</v>
+        <v>5.51</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>5.11</v>
+        <v>5.04</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>3.8</v>
+        <v>3.73</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>2.15</v>
+        <v>2.08</v>
       </c>
       <c r="H46" s="3" t="n">
         <v>0.17</v>
@@ -5126,19 +5126,19 @@
         <v>10.68</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>7.51</v>
+        <v>7.59</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>7.22</v>
+        <v>7.29</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>6.96</v>
+        <v>7.03</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>6.32</v>
+        <v>6.36</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>3.83</v>
+        <v>3.87</v>
       </c>
       <c r="H47" s="3" t="n">
         <v>0.67</v>
@@ -5157,7 +5157,7 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>6.22</v>
+        <v>5.95</v>
       </c>
       <c r="C48" s="3" t="n">
         <v>4.47</v>
@@ -5169,7 +5169,7 @@
         <v>3.09</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>0</v>
@@ -5191,7 +5191,7 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>13.58</v>
+        <v>13.51</v>
       </c>
       <c r="C49" s="3" t="n">
         <v>11.74</v>
@@ -5203,10 +5203,10 @@
         <v>9.859999999999999</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>7.36</v>
+        <v>7.29</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>4.03</v>
+        <v>3.99</v>
       </c>
       <c r="H49" s="3" t="n">
         <v>2.19</v>
@@ -5225,7 +5225,7 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>2.05</v>
+        <v>1.85</v>
       </c>
       <c r="C50" s="3" t="n">
         <v>1.34</v>
@@ -5259,7 +5259,7 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>4.72</v>
+        <v>4.44</v>
       </c>
       <c r="C51" s="3" t="n">
         <v>3.58</v>
@@ -5271,7 +5271,7 @@
         <v>2.71</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>2.15</v>
+        <v>1.84</v>
       </c>
       <c r="G51" s="3" t="n">
         <v>0.03</v>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>15.99</v>
+        <v>15.09</v>
       </c>
       <c r="C52" s="3" t="n">
         <v>12.6</v>
@@ -5305,7 +5305,7 @@
         <v>9.85</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="G52" s="3" t="n">
         <v>2.65</v>
@@ -5327,7 +5327,7 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>17.61</v>
+        <v>17.41</v>
       </c>
       <c r="C53" s="3" t="n">
         <v>14.01</v>
@@ -5339,7 +5339,7 @@
         <v>8.9</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>6.42</v>
+        <v>6.18</v>
       </c>
       <c r="G53" s="3" t="n">
         <v>1.85</v>
@@ -5361,22 +5361,22 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>39.27</v>
+        <v>39.03</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>35.62</v>
+        <v>35.42</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>32.81</v>
+        <v>32.64</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>25.62</v>
+        <v>25.52</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>24.24</v>
+        <v>24.13</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>16.88</v>
+        <v>16.84</v>
       </c>
       <c r="H54" s="3" t="n">
         <v>3.3</v>
@@ -5395,22 +5395,22 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>49.13</v>
+        <v>48.76</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>45.83</v>
+        <v>45.6</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>42.81</v>
+        <v>42.54</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>34.71</v>
+        <v>34.48</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>31.59</v>
+        <v>31.38</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>15.93</v>
+        <v>15.66</v>
       </c>
       <c r="H55" s="3" t="n">
         <v>1.61</v>
@@ -5429,19 +5429,19 @@
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>17.4</v>
+        <v>17.26</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>14.65</v>
+        <v>14.51</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>12.99</v>
+        <v>12.88</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>8.4</v>
+        <v>8.33</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>4.31</v>
+        <v>4.27</v>
       </c>
       <c r="G56" s="3" t="n">
         <v>1.35</v>
@@ -5463,19 +5463,19 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>21.24</v>
+        <v>21.2</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>19.76</v>
+        <v>19.72</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>15.83</v>
+        <v>15.76</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>12.16</v>
+        <v>12.1</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>6.82</v>
+        <v>6.85</v>
       </c>
       <c r="G57" s="3" t="n">
         <v>0.47</v>
@@ -5497,10 +5497,10 @@
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>4.64</v>
+        <v>4.6</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>3.83</v>
+        <v>3.8</v>
       </c>
       <c r="D58" s="3" t="n">
         <v>2.89</v>
@@ -5512,16 +5512,16 @@
         <v>1.04</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="H58" s="3" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="I58" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="I58" s="3" t="n">
+      <c r="J58" s="3" t="n">
         <v>0.37</v>
-      </c>
-      <c r="J58" s="3" t="n">
-        <v>0.34</v>
       </c>
     </row>
     <row r="59">
@@ -5531,16 +5531,16 @@
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>6.97</v>
+        <v>6.9</v>
       </c>
       <c r="C59" s="3" t="n">
-        <v>5.46</v>
+        <v>5.42</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>3.2</v>
+        <v>3.16</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1.83</v>
+        <v>1.8</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0.72</v>
@@ -5565,13 +5565,13 @@
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>13.78</v>
+        <v>13.61</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>11.29</v>
+        <v>11.16</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>8.199999999999999</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>4.23</v>
@@ -5599,19 +5599,19 @@
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>16.98</v>
+        <v>16.81</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>13.09</v>
+        <v>12.92</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>8.02</v>
+        <v>7.99</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>4.41</v>
+        <v>4.38</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>3.37</v>
+        <v>3.33</v>
       </c>
       <c r="G61" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -5667,7 +5667,7 @@
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>5.42</v>
+        <v>5.35</v>
       </c>
       <c r="C63" s="3" t="n">
         <v>3.99</v>
@@ -5704,7 +5704,7 @@
         <v>9.74</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>8.33</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>5.58</v>
@@ -5735,19 +5735,19 @@
         </is>
       </c>
       <c r="B65" s="3" t="n">
-        <v>30.71</v>
+        <v>30.54</v>
       </c>
       <c r="C65" s="3" t="n">
-        <v>27.45</v>
+        <v>27.28</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>24.9</v>
+        <v>24.76</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>22.01</v>
+        <v>21.98</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>18.58</v>
+        <v>18.55</v>
       </c>
       <c r="G65" s="3" t="n">
         <v>6.42</v>
@@ -5769,16 +5769,16 @@
         </is>
       </c>
       <c r="B66" s="3" t="n">
-        <v>56.7</v>
+        <v>56.67</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>50.97</v>
+        <v>50.94</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>48.54</v>
+        <v>48.51</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>44.06</v>
+        <v>44.03</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>36.6</v>
@@ -5803,19 +5803,19 @@
         </is>
       </c>
       <c r="B67" s="3" t="n">
-        <v>36.86</v>
+        <v>36.83</v>
       </c>
       <c r="C67" s="3" t="n">
-        <v>35.79</v>
+        <v>35.72</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>34.71</v>
+        <v>34.64</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>30.78</v>
+        <v>30.68</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>21.98</v>
+        <v>21.91</v>
       </c>
       <c r="G67" s="3" t="n">
         <v>4.77</v>
@@ -5837,16 +5837,16 @@
         </is>
       </c>
       <c r="B68" s="3" t="n">
-        <v>20.49</v>
+        <v>20.38</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>19.06</v>
+        <v>19.03</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>16.94</v>
+        <v>16.91</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>13.09</v>
+        <v>13.06</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>2.19</v>
@@ -5871,19 +5871,19 @@
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>36.29</v>
+        <v>36.12</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>34.44</v>
+        <v>34.27</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>31.18</v>
+        <v>31.01</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>23.66</v>
+        <v>23.49</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>3.49</v>
+        <v>3.46</v>
       </c>
       <c r="G69" s="3" t="n">
         <v>0.1</v>
@@ -5905,16 +5905,16 @@
         </is>
       </c>
       <c r="B70" s="3" t="n">
-        <v>35.32</v>
+        <v>35.22</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>34.17</v>
+        <v>34.11</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>29.87</v>
+        <v>29.84</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>19.42</v>
+        <v>19.35</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>1.34</v>
@@ -5939,16 +5939,16 @@
         </is>
       </c>
       <c r="B71" s="3" t="n">
-        <v>33.56</v>
+        <v>33.15</v>
       </c>
       <c r="C71" s="3" t="n">
-        <v>32.07</v>
+        <v>31.85</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>29.72</v>
+        <v>29.58</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>17.97</v>
+        <v>17.82</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>2.38</v>
@@ -5973,16 +5973,16 @@
         </is>
       </c>
       <c r="B72" s="3" t="n">
-        <v>23.66</v>
+        <v>23.15</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>19.79</v>
+        <v>19.56</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>15.93</v>
+        <v>15.73</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.54</v>
+        <v>0.5</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0.1</v>
@@ -6007,16 +6007,16 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>30.52</v>
+        <v>30.03</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>26.6</v>
+        <v>26.39</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>21.84</v>
+        <v>21.7</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>4.65</v>
+        <v>4.55</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0</v>
@@ -6041,13 +6041,13 @@
         </is>
       </c>
       <c r="B74" s="3" t="n">
-        <v>19.96</v>
+        <v>19.56</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>17.91</v>
+        <v>17.84</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>11.66</v>
+        <v>11.63</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>0.03</v>
@@ -6075,10 +6075,10 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>7.99</v>
+        <v>7.85</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>6.46</v>
+        <v>6.42</v>
       </c>
       <c r="D75" s="3" t="n">
         <v>2.33</v>
@@ -6109,13 +6109,13 @@
         </is>
       </c>
       <c r="B76" s="3" t="n">
-        <v>15.66</v>
+        <v>15.52</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>11.76</v>
+        <v>11.69</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>1.75</v>
+        <v>1.71</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>0</v>
@@ -6143,10 +6143,10 @@
         </is>
       </c>
       <c r="B77" s="3" t="n">
-        <v>26.88</v>
+        <v>26.75</v>
       </c>
       <c r="C77" s="3" t="n">
-        <v>19.29</v>
+        <v>19.32</v>
       </c>
       <c r="D77" s="3" t="n">
         <v>1.58</v>
@@ -6177,10 +6177,10 @@
         </is>
       </c>
       <c r="B78" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>70.62</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>60.73</v>
+        <v>60.56</v>
       </c>
       <c r="D78" s="3" t="n">
         <v>15.49</v>
@@ -6211,10 +6211,10 @@
         </is>
       </c>
       <c r="B79" s="3" t="n">
-        <v>59.85</v>
+        <v>59.48</v>
       </c>
       <c r="C79" s="3" t="n">
-        <v>48.62</v>
+        <v>48.45</v>
       </c>
       <c r="D79" s="3" t="n">
         <v>17.27</v>
@@ -6245,31 +6245,31 @@
         </is>
       </c>
       <c r="B80" s="3" t="n">
-        <v>74.72</v>
+        <v>74.41</v>
       </c>
       <c r="C80" s="3" t="n">
-        <v>53.85</v>
+        <v>53.33</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>15.97</v>
+        <v>16.04</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>3.99</v>
+        <v>4.03</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>1.39</v>
+        <v>1.42</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="81">
@@ -6279,13 +6279,13 @@
         </is>
       </c>
       <c r="B81" s="3" t="n">
-        <v>49.97</v>
+        <v>48.89</v>
       </c>
       <c r="C81" s="3" t="n">
-        <v>23.12</v>
+        <v>22.88</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>7.02</v>
+        <v>6.99</v>
       </c>
       <c r="E81" s="3" t="n">
         <v>4.33</v>
@@ -6313,16 +6313,16 @@
         </is>
       </c>
       <c r="B82" s="3" t="n">
-        <v>18.04</v>
+        <v>16.3</v>
       </c>
       <c r="C82" s="3" t="n">
-        <v>2.65</v>
+        <v>2.69</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F82" s="3" t="n">
         <v>0.1</v>
@@ -6347,16 +6347,16 @@
         </is>
       </c>
       <c r="B83" s="3" t="n">
-        <v>10.04</v>
+        <v>10.12</v>
       </c>
       <c r="C83" s="3" t="n">
-        <v>1.6</v>
+        <v>1.64</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>0.04</v>
@@ -6381,7 +6381,7 @@
         </is>
       </c>
       <c r="B84" s="3" t="n">
-        <v>13.51</v>
+        <v>13.27</v>
       </c>
       <c r="C84" s="3" t="n">
         <v>0.27</v>
@@ -6415,7 +6415,7 @@
         </is>
       </c>
       <c r="B85" s="3" t="n">
-        <v>19.2</v>
+        <v>18.78</v>
       </c>
       <c r="C85" s="3" t="n">
         <v>2.15</v>
@@ -6449,7 +6449,7 @@
         </is>
       </c>
       <c r="B86" s="3" t="n">
-        <v>4.3</v>
+        <v>4.03</v>
       </c>
       <c r="C86" s="3" t="n">
         <v>0</v>
@@ -6483,7 +6483,7 @@
         </is>
       </c>
       <c r="B87" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="C87" s="3" t="n">
         <v>0</v>
@@ -6517,7 +6517,7 @@
         </is>
       </c>
       <c r="B88" s="3" t="n">
-        <v>4.37</v>
+        <v>4.33</v>
       </c>
       <c r="C88" s="3" t="n">
         <v>0</v>
@@ -6551,7 +6551,7 @@
         </is>
       </c>
       <c r="B89" s="3" t="n">
-        <v>6.92</v>
+        <v>6.82</v>
       </c>
       <c r="C89" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -6817,7 +6817,7 @@
         <v>2880</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>0</v>
@@ -6854,7 +6854,7 @@
         <v>2976</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>0</v>
@@ -6891,7 +6891,7 @@
         <v>2976</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>3</v>
@@ -6928,7 +6928,7 @@
         <v>2880</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>5</v>
@@ -6965,7 +6965,7 @@
         <v>2976</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>3</v>
@@ -7076,10 +7076,10 @@
         <v>2976</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>3</v>
@@ -7113,7 +7113,7 @@
         <v>2784</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -7150,7 +7150,7 @@
         <v>2976</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
@@ -7187,7 +7187,7 @@
         <v>2880</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>36</v>
@@ -7224,7 +7224,7 @@
         <v>2976</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>0</v>
@@ -7298,7 +7298,7 @@
         <v>2976</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>4</v>
@@ -7335,7 +7335,7 @@
         <v>2976</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>2</v>
@@ -7372,7 +7372,7 @@
         <v>2880</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>1</v>
@@ -7409,7 +7409,7 @@
         <v>2976</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19" s="6" t="n">
         <v>2</v>
@@ -7594,7 +7594,7 @@
         <v>2976</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D24" s="6" t="n">
         <v>0</v>
@@ -7631,7 +7631,7 @@
         <v>2880</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>75</v>
@@ -7668,7 +7668,7 @@
         <v>2976</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>5</v>
@@ -7705,7 +7705,7 @@
         <v>2880</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="6" t="n">
         <v>1</v>
@@ -7742,31 +7742,31 @@
         <v>2976</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -7779,19 +7779,19 @@
         <v>2976</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H29" s="6" t="n">
         <v>36</v>
@@ -7816,16 +7816,16 @@
         <v>2880</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>781</v>
+        <v>766</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>74</v>
@@ -7853,10 +7853,10 @@
         <v>2976</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>722</v>
+        <v>716</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E31" s="6" t="n">
         <v>538</v>
@@ -7890,16 +7890,16 @@
         <v>2880</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>28</v>
@@ -7927,13 +7927,13 @@
         <v>2976</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>73</v>
@@ -7964,7 +7964,7 @@
         <v>2976</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D34" s="6" t="n">
         <v>7</v>
@@ -8001,10 +8001,10 @@
         <v>2688</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E35" s="6" t="n">
         <v>53</v>
@@ -8038,7 +8038,7 @@
         <v>2976</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="6" t="n">
         <v>2</v>
@@ -8075,7 +8075,7 @@
         <v>2880</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D37" s="6" t="n">
         <v>4</v>
@@ -8149,7 +8149,7 @@
         <v>2880</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D39" s="6" t="n">
         <v>17</v>
@@ -8186,7 +8186,7 @@
         <v>2976</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D40" s="6" t="n">
         <v>28</v>
@@ -8223,13 +8223,13 @@
         <v>2976</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D41" s="6" t="n">
         <v>170</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>140</v>
@@ -8260,10 +8260,10 @@
         <v>2880</v>
       </c>
       <c r="C42" s="6" t="n">
-        <v>541</v>
+        <v>536</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="E42" s="6" t="n">
         <v>427</v>
@@ -8278,10 +8278,10 @@
         <v>167</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K42" s="6" t="n">
         <v>0</v>
@@ -8297,25 +8297,25 @@
         <v>2976</v>
       </c>
       <c r="C43" s="6" t="n">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J43" s="6" t="n">
         <v>30</v>
@@ -8334,25 +8334,25 @@
         <v>2880</v>
       </c>
       <c r="C44" s="6" t="n">
-        <v>593</v>
+        <v>587</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J44" s="6" t="n">
         <v>11</v>
@@ -8371,22 +8371,22 @@
         <v>2976</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>658</v>
+        <v>649</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>579</v>
+        <v>570</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="I45" s="6" t="n">
         <v>56</v>
@@ -8408,22 +8408,22 @@
         <v>2976</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>5</v>
@@ -8448,19 +8448,19 @@
         <v>287</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I47" s="6" t="n">
         <v>18</v>
@@ -8482,7 +8482,7 @@
         <v>2976</v>
       </c>
       <c r="C48" s="6" t="n">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D48" s="6" t="n">
         <v>133</v>
@@ -8494,7 +8494,7 @@
         <v>92</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H48" s="6" t="n">
         <v>0</v>
@@ -8519,7 +8519,7 @@
         <v>2880</v>
       </c>
       <c r="C49" s="6" t="n">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D49" s="6" t="n">
         <v>338</v>
@@ -8531,10 +8531,10 @@
         <v>284</v>
       </c>
       <c r="G49" s="6" t="n">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>63</v>
@@ -8556,7 +8556,7 @@
         <v>2976</v>
       </c>
       <c r="C50" s="6" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D50" s="6" t="n">
         <v>40</v>
@@ -8593,7 +8593,7 @@
         <v>2880</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D51" s="6" t="n">
         <v>103</v>
@@ -8605,7 +8605,7 @@
         <v>78</v>
       </c>
       <c r="G51" s="6" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="H51" s="6" t="n">
         <v>1</v>
@@ -8630,7 +8630,7 @@
         <v>2976</v>
       </c>
       <c r="C52" s="6" t="n">
-        <v>476</v>
+        <v>449</v>
       </c>
       <c r="D52" s="6" t="n">
         <v>375</v>
@@ -8642,7 +8642,7 @@
         <v>293</v>
       </c>
       <c r="G52" s="6" t="n">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="H52" s="6" t="n">
         <v>79</v>
@@ -8667,7 +8667,7 @@
         <v>2976</v>
       </c>
       <c r="C53" s="6" t="n">
-        <v>524</v>
+        <v>518</v>
       </c>
       <c r="D53" s="6" t="n">
         <v>417</v>
@@ -8679,7 +8679,7 @@
         <v>265</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="H53" s="6" t="n">
         <v>55</v>
@@ -8704,22 +8704,22 @@
         <v>2880</v>
       </c>
       <c r="C54" s="6" t="n">
-        <v>1131</v>
+        <v>1124</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="F54" s="6" t="n">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="I54" s="6" t="n">
         <v>95</v>
@@ -8741,22 +8741,22 @@
         <v>2976</v>
       </c>
       <c r="C55" s="6" t="n">
-        <v>1462</v>
+        <v>1451</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>1364</v>
+        <v>1357</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>1274</v>
+        <v>1266</v>
       </c>
       <c r="F55" s="6" t="n">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="G55" s="6" t="n">
-        <v>940</v>
+        <v>934</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="I55" s="6" t="n">
         <v>48</v>
@@ -8778,19 +8778,19 @@
         <v>2880</v>
       </c>
       <c r="C56" s="6" t="n">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="F56" s="6" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="G56" s="6" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H56" s="6" t="n">
         <v>39</v>
@@ -8815,19 +8815,19 @@
         <v>2976</v>
       </c>
       <c r="C57" s="6" t="n">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="F57" s="6" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H57" s="6" t="n">
         <v>14</v>
@@ -8852,10 +8852,10 @@
         <v>2976</v>
       </c>
       <c r="C58" s="6" t="n">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E58" s="6" t="n">
         <v>86</v>
@@ -8867,16 +8867,16 @@
         <v>31</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I58" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J58" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J58" s="6" t="n">
+      <c r="K58" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="K58" s="6" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="59">
@@ -8889,16 +8889,16 @@
         <v>2784</v>
       </c>
       <c r="C59" s="6" t="n">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G59" s="6" t="n">
         <v>20</v>
@@ -8926,13 +8926,13 @@
         <v>2976</v>
       </c>
       <c r="C60" s="6" t="n">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="F60" s="6" t="n">
         <v>126</v>
@@ -8963,19 +8963,19 @@
         <v>2880</v>
       </c>
       <c r="C61" s="6" t="n">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G61" s="6" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H61" s="6" t="n">
         <v>2</v>
@@ -9037,7 +9037,7 @@
         <v>2880</v>
       </c>
       <c r="C63" s="6" t="n">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D63" s="6" t="n">
         <v>115</v>
@@ -9077,7 +9077,7 @@
         <v>290</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E64" s="6" t="n">
         <v>166</v>
@@ -9111,19 +9111,19 @@
         <v>2976</v>
       </c>
       <c r="C65" s="6" t="n">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="G65" s="6" t="n">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>191</v>
@@ -9148,16 +9148,16 @@
         <v>2880</v>
       </c>
       <c r="C66" s="6" t="n">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="F66" s="6" t="n">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="G66" s="6" t="n">
         <v>1054</v>
@@ -9185,19 +9185,19 @@
         <v>2976</v>
       </c>
       <c r="C67" s="6" t="n">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="F67" s="6" t="n">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="G67" s="6" t="n">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="H67" s="6" t="n">
         <v>142</v>
@@ -9222,16 +9222,16 @@
         <v>2880</v>
       </c>
       <c r="C68" s="6" t="n">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F68" s="6" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G68" s="6" t="n">
         <v>63</v>
@@ -9259,19 +9259,19 @@
         <v>2976</v>
       </c>
       <c r="C69" s="6" t="n">
-        <v>1080</v>
+        <v>1075</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>1025</v>
+        <v>1020</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>704</v>
+        <v>699</v>
       </c>
       <c r="G69" s="6" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H69" s="6" t="n">
         <v>3</v>
@@ -9296,16 +9296,16 @@
         <v>2976</v>
       </c>
       <c r="C70" s="6" t="n">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="F70" s="6" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="G70" s="6" t="n">
         <v>40</v>
@@ -9333,16 +9333,16 @@
         <v>2688</v>
       </c>
       <c r="C71" s="6" t="n">
-        <v>902</v>
+        <v>891</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>862</v>
+        <v>856</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="G71" s="6" t="n">
         <v>64</v>
@@ -9370,16 +9370,16 @@
         <v>2976</v>
       </c>
       <c r="C72" s="6" t="n">
-        <v>704</v>
+        <v>689</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>589</v>
+        <v>582</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G72" s="6" t="n">
         <v>3</v>
@@ -9407,16 +9407,16 @@
         <v>2880</v>
       </c>
       <c r="C73" s="6" t="n">
-        <v>879</v>
+        <v>865</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G73" s="6" t="n">
         <v>0</v>
@@ -9444,13 +9444,13 @@
         <v>2976</v>
       </c>
       <c r="C74" s="6" t="n">
-        <v>594</v>
+        <v>582</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F74" s="6" t="n">
         <v>1</v>
@@ -9481,10 +9481,10 @@
         <v>2880</v>
       </c>
       <c r="C75" s="6" t="n">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E75" s="6" t="n">
         <v>67</v>
@@ -9518,13 +9518,13 @@
         <v>2976</v>
       </c>
       <c r="C76" s="6" t="n">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F76" s="6" t="n">
         <v>0</v>
@@ -9555,10 +9555,10 @@
         <v>2976</v>
       </c>
       <c r="C77" s="6" t="n">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E77" s="6" t="n">
         <v>47</v>
@@ -9592,10 +9592,10 @@
         <v>2880</v>
       </c>
       <c r="C78" s="6" t="n">
-        <v>2042</v>
+        <v>2034</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>1749</v>
+        <v>1744</v>
       </c>
       <c r="E78" s="6" t="n">
         <v>446</v>
@@ -9629,10 +9629,10 @@
         <v>2976</v>
       </c>
       <c r="C79" s="6" t="n">
-        <v>1781</v>
+        <v>1770</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>1447</v>
+        <v>1442</v>
       </c>
       <c r="E79" s="6" t="n">
         <v>514</v>
@@ -9666,31 +9666,31 @@
         <v>2880</v>
       </c>
       <c r="C80" s="6" t="n">
-        <v>2152</v>
+        <v>2143</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>1551</v>
+        <v>1536</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G80" s="6" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H80" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I80" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J80" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K80" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81">
@@ -9703,13 +9703,13 @@
         <v>2976</v>
       </c>
       <c r="C81" s="6" t="n">
-        <v>1487</v>
+        <v>1455</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>688</v>
+        <v>681</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F81" s="6" t="n">
         <v>129</v>
@@ -9740,16 +9740,16 @@
         <v>2976</v>
       </c>
       <c r="C82" s="6" t="n">
-        <v>537</v>
+        <v>485</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F82" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G82" s="6" t="n">
         <v>3</v>
@@ -9777,16 +9777,16 @@
         <v>2688</v>
       </c>
       <c r="C83" s="6" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G83" s="6" t="n">
         <v>1</v>
@@ -9814,7 +9814,7 @@
         <v>2976</v>
       </c>
       <c r="C84" s="6" t="n">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="D84" s="6" t="n">
         <v>8</v>
@@ -9851,7 +9851,7 @@
         <v>2880</v>
       </c>
       <c r="C85" s="6" t="n">
-        <v>553</v>
+        <v>541</v>
       </c>
       <c r="D85" s="6" t="n">
         <v>62</v>
@@ -9888,7 +9888,7 @@
         <v>2976</v>
       </c>
       <c r="C86" s="6" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D86" s="6" t="n">
         <v>0</v>
@@ -9925,7 +9925,7 @@
         <v>2880</v>
       </c>
       <c r="C87" s="6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D87" s="6" t="n">
         <v>0</v>
@@ -9962,7 +9962,7 @@
         <v>2976</v>
       </c>
       <c r="C88" s="6" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D88" s="6" t="n">
         <v>0</v>
@@ -9999,7 +9999,7 @@
         <v>2976</v>
       </c>
       <c r="C89" s="6" t="n">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D89" s="6" t="n">
         <v>2</v>

</xml_diff>